<commit_message>
added weight dropdown 70g and 100g with price update
</commit_message>
<xml_diff>
--- a/public/soaps.xlsx
+++ b/public/soaps.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,21 +407,24 @@
         <v>description</v>
       </c>
       <c r="C1" t="str">
-        <v>price</v>
+        <v>price100g</v>
       </c>
       <c r="D1" t="str">
-        <v>weight</v>
+        <v>price70g</v>
       </c>
       <c r="E1" t="str">
-        <v>inStock</v>
+        <v>inStock100g</v>
       </c>
       <c r="F1" t="str">
+        <v>inStock70g</v>
+      </c>
+      <c r="G1" t="str">
         <v>image1</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>image2</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>image3</v>
       </c>
     </row>
@@ -433,22 +436,25 @@
         <v>Traditional herbal soap made with Kuppameni leaves for healthy skin</v>
       </c>
       <c r="C2">
-        <v>120</v>
-      </c>
-      <c r="D2" t="str">
-        <v>100g</v>
+        <v>100</v>
+      </c>
+      <c r="D2">
+        <v>50</v>
       </c>
       <c r="E2" t="str">
         <v>yes</v>
       </c>
       <c r="F2" t="str">
-        <v>/images/kuppameni1.jpg</v>
+        <v>yes</v>
       </c>
       <c r="G2" t="str">
-        <v>/images/kuppameni2.jpg</v>
+        <v>/images/kuppameni1.jpeg</v>
       </c>
       <c r="H2" t="str">
-        <v>/images/kuppameni3.jpg</v>
+        <v>/images/kuppameni2.jpeg</v>
+      </c>
+      <c r="I2" t="str">
+        <v>/images/kuppameni3.jpeg</v>
       </c>
     </row>
     <row r="3">
@@ -459,22 +465,25 @@
         <v>Skin brightening soap with natural papaya extract</v>
       </c>
       <c r="C3">
-        <v>130</v>
-      </c>
-      <c r="D3" t="str">
-        <v>100g</v>
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>50</v>
       </c>
       <c r="E3" t="str">
         <v>yes</v>
       </c>
       <c r="F3" t="str">
-        <v>/images/papaya1.jpg</v>
+        <v>yes</v>
       </c>
       <c r="G3" t="str">
-        <v>/images/papaya2.jpg</v>
+        <v>/images/papaya1.jpeg</v>
       </c>
       <c r="H3" t="str">
-        <v>/images/papaya3.jpg</v>
+        <v>/images/papaya2.jpeg</v>
+      </c>
+      <c r="I3" t="str">
+        <v>/images/papaya3.jpeg</v>
       </c>
     </row>
     <row r="4">
@@ -485,22 +494,25 @@
         <v>Moisturizing soap with fresh aloe vera gel</v>
       </c>
       <c r="C4">
-        <v>110</v>
-      </c>
-      <c r="D4" t="str">
-        <v>100g</v>
+        <v>100</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
       </c>
       <c r="E4" t="str">
         <v>yes</v>
       </c>
       <c r="F4" t="str">
-        <v>/images/aloevera1.jpg</v>
+        <v>yes</v>
       </c>
       <c r="G4" t="str">
-        <v>/images/aloevera2.jpg</v>
+        <v>/images/aloevera1.jpeg</v>
       </c>
       <c r="H4" t="str">
-        <v>/images/aloevera3.jpg</v>
+        <v>/images/aloevera2.jpeg</v>
+      </c>
+      <c r="I4" t="str">
+        <v>/images/aloevera3.jpeg</v>
       </c>
     </row>
     <row r="5">
@@ -511,27 +523,30 @@
         <v>Deep cleansing activated charcoal soap for oil control</v>
       </c>
       <c r="C5">
-        <v>140</v>
-      </c>
-      <c r="D5" t="str">
-        <v>100g</v>
+        <v>100</v>
+      </c>
+      <c r="D5">
+        <v>50</v>
       </c>
       <c r="E5" t="str">
         <v>yes</v>
       </c>
       <c r="F5" t="str">
-        <v>/images/charcoal1.jpg</v>
+        <v>yes</v>
       </c>
       <c r="G5" t="str">
-        <v>/images/charcoal2.jpg</v>
+        <v>/images/charcoal1.jpeg</v>
       </c>
       <c r="H5" t="str">
-        <v>/images/charcoal3.jpg</v>
+        <v>/images/charcoal2.jpeg</v>
+      </c>
+      <c r="I5" t="str">
+        <v>/images/charcoal3.jpeg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added Acne Clear Soap
</commit_message>
<xml_diff>
--- a/public/soaps.xlsx
+++ b/public/soaps.xlsx
@@ -1,41 +1,133 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects_K\vanam-soaps\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="10800"/>
+  </bookViews>
   <sheets>
     <sheet name="Soaps" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>price100g</t>
+  </si>
+  <si>
+    <t>price70g</t>
+  </si>
+  <si>
+    <t>inStock100g</t>
+  </si>
+  <si>
+    <t>inStock70g</t>
+  </si>
+  <si>
+    <t>image1</t>
+  </si>
+  <si>
+    <t>image2</t>
+  </si>
+  <si>
+    <t>image3</t>
+  </si>
+  <si>
+    <t>Kuppameni Soap</t>
+  </si>
+  <si>
+    <t>Traditional herbal soap made with Kuppameni leaves for healthy skin</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>/images/kuppameni1.jpeg</t>
+  </si>
+  <si>
+    <t>/images/kuppameni2.jpeg</t>
+  </si>
+  <si>
+    <t>/images/kuppameni3.jpeg</t>
+  </si>
+  <si>
+    <t>Papaya Soap</t>
+  </si>
+  <si>
+    <t>Skin brightening soap with natural papaya extract</t>
+  </si>
+  <si>
+    <t>/images/papaya1.jpeg</t>
+  </si>
+  <si>
+    <t>/images/papaya2.jpeg</t>
+  </si>
+  <si>
+    <t>/images/papaya3.jpeg</t>
+  </si>
+  <si>
+    <t>Aloe Vera Soap</t>
+  </si>
+  <si>
+    <t>Moisturizing soap with fresh aloe vera gel</t>
+  </si>
+  <si>
+    <t>/images/aloevera1.jpeg</t>
+  </si>
+  <si>
+    <t>/images/aloevera2.jpeg</t>
+  </si>
+  <si>
+    <t>/images/aloevera3.jpeg</t>
+  </si>
+  <si>
+    <t>Charcoal Soap</t>
+  </si>
+  <si>
+    <t>Deep cleansing activated charcoal soap for oil control</t>
+  </si>
+  <si>
+    <t>/images/charcoal1.jpeg</t>
+  </si>
+  <si>
+    <t>/images/charcoal2.jpeg</t>
+  </si>
+  <si>
+    <t>/images/charcoal3.jpeg</t>
+  </si>
+  <si>
+    <t>Deep cleansing , Moisturizing soap for acne and oil control</t>
+  </si>
+  <si>
+    <t>/images/acnesoap1.jpeg</t>
+  </si>
+  <si>
+    <t>/images/acnesoap2.jpeg</t>
+  </si>
+  <si>
+    <t>/images/acnesoap3.jpeg</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -72,6 +164,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,44 +496,52 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="22.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>description</v>
-      </c>
-      <c r="C1" t="str">
-        <v>price100g</v>
-      </c>
-      <c r="D1" t="str">
-        <v>price70g</v>
-      </c>
-      <c r="E1" t="str">
-        <v>inStock100g</v>
-      </c>
-      <c r="F1" t="str">
-        <v>inStock70g</v>
-      </c>
-      <c r="G1" t="str">
-        <v>image1</v>
-      </c>
-      <c r="H1" t="str">
-        <v>image2</v>
-      </c>
-      <c r="I1" t="str">
-        <v>image3</v>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Kuppameni Soap</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Traditional herbal soap made with Kuppameni leaves for healthy skin</v>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -441,28 +549,28 @@
       <c r="D2">
         <v>50</v>
       </c>
-      <c r="E2" t="str">
-        <v>yes</v>
-      </c>
-      <c r="F2" t="str">
-        <v>yes</v>
-      </c>
-      <c r="G2" t="str">
-        <v>/images/kuppameni1.jpeg</v>
-      </c>
-      <c r="H2" t="str">
-        <v>/images/kuppameni2.jpeg</v>
-      </c>
-      <c r="I2" t="str">
-        <v>/images/kuppameni3.jpeg</v>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Papaya Soap</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Skin brightening soap with natural papaya extract</v>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -470,28 +578,28 @@
       <c r="D3">
         <v>50</v>
       </c>
-      <c r="E3" t="str">
-        <v>yes</v>
-      </c>
-      <c r="F3" t="str">
-        <v>yes</v>
-      </c>
-      <c r="G3" t="str">
-        <v>/images/papaya1.jpeg</v>
-      </c>
-      <c r="H3" t="str">
-        <v>/images/papaya2.jpeg</v>
-      </c>
-      <c r="I3" t="str">
-        <v>/images/papaya3.jpeg</v>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Aloe Vera Soap</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Moisturizing soap with fresh aloe vera gel</v>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -499,28 +607,28 @@
       <c r="D4">
         <v>50</v>
       </c>
-      <c r="E4" t="str">
-        <v>yes</v>
-      </c>
-      <c r="F4" t="str">
-        <v>yes</v>
-      </c>
-      <c r="G4" t="str">
-        <v>/images/aloevera1.jpeg</v>
-      </c>
-      <c r="H4" t="str">
-        <v>/images/aloevera2.jpeg</v>
-      </c>
-      <c r="I4" t="str">
-        <v>/images/aloevera3.jpeg</v>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Charcoal Soap</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Deep cleansing activated charcoal soap for oil control</v>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -528,25 +636,55 @@
       <c r="D5">
         <v>50</v>
       </c>
-      <c r="E5" t="str">
-        <v>yes</v>
-      </c>
-      <c r="F5" t="str">
-        <v>yes</v>
-      </c>
-      <c r="G5" t="str">
-        <v>/images/charcoal1.jpeg</v>
-      </c>
-      <c r="H5" t="str">
-        <v>/images/charcoal2.jpeg</v>
-      </c>
-      <c r="I5" t="str">
-        <v>/images/charcoal3.jpeg</v>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6">
+        <v>120</v>
+      </c>
+      <c r="D6">
+        <v>100</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError sqref="A1:I3 A5:I5 A4 C4:I4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>